<commit_message>
add cyntec hbed063t inductors
</commit_message>
<xml_diff>
--- a/data/cyntec_inductor_data.xlsx
+++ b/data/cyntec_inductor_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://renesasgroup-my.sharepoint.com/personal/gary_kidwell_wz_renesas_com/Documents/python/charger/mathmodels/pdis_2or3lvl_bb/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="803" documentId="11_88A5EEC595FCDE19E65C93C75DD0486FD8C93E14" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{160B5F0C-4B7F-4577-AABA-9F5AB12CA9CB}"/>
+  <xr:revisionPtr revIDLastSave="825" documentId="11_88A5EEC595FCDE19E65C93C75DD0486FD8C93E14" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D6DCF0E-86A3-46A6-8FCA-F55B26DF33DD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="772" firstSheet="11" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29910" yWindow="1620" windowWidth="21000" windowHeight="12735" tabRatio="772" firstSheet="11" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="htel20121b" sheetId="21" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="39">
   <si>
     <t>Lout</t>
   </si>
@@ -2138,7 +2138,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40693CA2-7319-4057-AD3C-7C4101A3AA7E}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="7" max="7" width="10.28515625" bestFit="1" customWidth="1"/>
@@ -2190,30 +2190,30 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>2.2000000000000002</v>
+        <v>0.47</v>
       </c>
       <c r="B2">
-        <v>1.0699999999999999E-2</v>
+        <v>2E-3</v>
       </c>
       <c r="C2">
-        <v>11.5</v>
+        <v>24</v>
       </c>
       <c r="D2">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="E2" s="2">
-        <f t="shared" ref="E2" si="0">40/F2</f>
-        <v>24.580046072223862</v>
+        <f t="shared" ref="E2:E4" si="0">40/F2</f>
+        <v>30.193236714975846</v>
       </c>
       <c r="F2" s="1">
-        <f t="shared" ref="F2" si="1">C2^2*B2*1.15</f>
-        <v>1.6273362499999997</v>
-      </c>
-      <c r="G2">
-        <v>1.3499999999999999E-5</v>
-      </c>
-      <c r="H2">
-        <v>1.3480000000000001E-2</v>
+        <f t="shared" ref="F2:F4" si="1">C2^2*B2*1.15</f>
+        <v>1.3248</v>
+      </c>
+      <c r="G2" s="3">
+        <v>1.489E-5</v>
+      </c>
+      <c r="H2" s="3">
+        <v>6.3949999999999996E-3</v>
       </c>
       <c r="I2">
         <v>1.254</v>
@@ -2231,6 +2231,98 @@
         <v>6.8</v>
       </c>
       <c r="N2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>0.68</v>
+      </c>
+      <c r="B3">
+        <v>2.7000000000000001E-3</v>
+      </c>
+      <c r="C3">
+        <v>20.7</v>
+      </c>
+      <c r="D3">
+        <v>25.5</v>
+      </c>
+      <c r="E3" s="2">
+        <f t="shared" si="0"/>
+        <v>30.064756855600741</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" si="1"/>
+        <v>1.3304614499999998</v>
+      </c>
+      <c r="G3" s="3">
+        <v>1.3159999999999999E-5</v>
+      </c>
+      <c r="H3" s="3">
+        <v>9.3860000000000002E-3</v>
+      </c>
+      <c r="I3">
+        <v>1.254</v>
+      </c>
+      <c r="J3">
+        <v>2.3260000000000001</v>
+      </c>
+      <c r="K3" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3">
+        <v>8.4</v>
+      </c>
+      <c r="M3">
+        <v>6.8</v>
+      </c>
+      <c r="N3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B4">
+        <v>1.0699999999999999E-2</v>
+      </c>
+      <c r="C4">
+        <v>11.5</v>
+      </c>
+      <c r="D4">
+        <v>18</v>
+      </c>
+      <c r="E4" s="2">
+        <f t="shared" si="0"/>
+        <v>24.580046072223862</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="1"/>
+        <v>1.6273362499999997</v>
+      </c>
+      <c r="G4">
+        <v>1.3499999999999999E-5</v>
+      </c>
+      <c r="H4">
+        <v>1.3480000000000001E-2</v>
+      </c>
+      <c r="I4">
+        <v>1.254</v>
+      </c>
+      <c r="J4">
+        <v>2.3260000000000001</v>
+      </c>
+      <c r="K4" t="s">
+        <v>28</v>
+      </c>
+      <c r="L4">
+        <v>8.4</v>
+      </c>
+      <c r="M4">
+        <v>6.8</v>
+      </c>
+      <c r="N4">
         <v>3</v>
       </c>
     </row>

</xml_diff>